<commit_message>
Update: Novotel-March-2026 by superadmin
</commit_message>
<xml_diff>
--- a/Novotel-March-2026.xlsx
+++ b/Novotel-March-2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\2023031\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7DEE3FC-647F-4503-A81E-60C6E841C169}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60C9D105-C7F6-4DDC-9415-51FDE5D5AA68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{E82819E8-EFF0-4774-BA8F-CEEEEB2C50F6}"/>
   </bookViews>
@@ -656,8 +656,8 @@
         <v>15</v>
       </c>
       <c r="G2" s="1">
-        <f t="shared" ref="G2:G9" ca="1" si="0">TODAY()-RANDBETWEEN(365,365*5)</f>
-        <v>45167</v>
+        <f ca="1">TODAY()-RANDBETWEEN(365,365*2)</f>
+        <v>45460</v>
       </c>
       <c r="H2">
         <v>79190</v>
@@ -737,8 +737,8 @@
         <v>15</v>
       </c>
       <c r="G3" s="1">
-        <f t="shared" ca="1" si="0"/>
-        <v>45012</v>
+        <f t="shared" ref="G3:G9" ca="1" si="0">TODAY()-RANDBETWEEN(365,365*2)</f>
+        <v>45663</v>
       </c>
       <c r="H3">
         <v>76180</v>
@@ -819,7 +819,7 @@
       </c>
       <c r="G4" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44656</v>
+        <v>45649</v>
       </c>
       <c r="H4">
         <v>93327</v>
@@ -900,7 +900,7 @@
       </c>
       <c r="G5" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44788</v>
+        <v>45518</v>
       </c>
       <c r="H5">
         <v>102201</v>
@@ -981,7 +981,7 @@
       </c>
       <c r="G6" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>45493</v>
+        <v>45471</v>
       </c>
       <c r="H6">
         <v>95486</v>
@@ -1062,7 +1062,7 @@
       </c>
       <c r="G7" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>45784</v>
+        <v>45429</v>
       </c>
       <c r="H7">
         <v>98229</v>
@@ -1143,7 +1143,7 @@
       </c>
       <c r="G8" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>44375</v>
+        <v>45583</v>
       </c>
       <c r="H8">
         <v>88062</v>
@@ -1224,7 +1224,7 @@
       </c>
       <c r="G9" s="1">
         <f t="shared" ca="1" si="0"/>
-        <v>45383</v>
+        <v>45730</v>
       </c>
       <c r="H9">
         <v>101386</v>

</xml_diff>